<commit_message>
Land PLTU Suralaya Unit 3 on the bus the book draws it on
Gambar 2.3 puts Unit 3 at the far left of TIER-1 with its own step-up
dropping onto the 150 kV Suralaya bus. The fixture had its outlet on
SRLYABR, the 500 kV GITET, so the generator hung off the wrong side of
the transformation and its lead never reached the 150 kV bus the figure
shows it feeding.

Point the outlet at SRLYA and register the unit at 150 kV.

SS_SLCG only; no other subsystem's registration is touched.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/ss_slcg_ingest.xlsx
+++ b/samples/ss_slcg_ingest.xlsx
@@ -788,7 +788,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>500 kV</t>
+          <t>150 kV</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -1578,12 +1578,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SRLYABR</t>
+          <t>SRLYA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>500 kV</t>
+          <t>150 kV</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>

</xml_diff>